<commit_message>
Rename "focus areas" to "Projects" and simplify content forms
- Website: research content collection renamed research → projects;
  Research page heading, eyebrows, and homepage section now say
  "Projects" (nav item stays "Research"). Same 3-item structure.
- Member Word form simplified to three short sections plus a PI block,
  with a 3-4 sentence "A bit about you" field for personality and
  "Project(s)" wording.
- Workbook: "Research Areas" sheet → "Projects", "Research area"
  column → "Project".
- Importer updated to the new sheet/column/folder names, and its
  example-row detection tightened to a per-sheet key column so a real
  publication tagged with an example project name is no longer skipped.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content-forms/Kuo-Lab-Content-Workbook.xlsx
+++ b/content-forms/Kuo-Lab-Content-Workbook.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Publications" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Alumni" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="News" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Research Areas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Projects" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -551,7 +551,7 @@
       </c>
       <c r="F5" s="4" t="inlineStr">
         <is>
-          <t>Research area</t>
+          <t>Project</t>
         </is>
       </c>
       <c r="G5" s="4" t="inlineStr">
@@ -598,7 +598,7 @@
       </c>
       <c r="F6" s="5" t="inlineStr">
         <is>
-          <t>Which focus area it belongs to</t>
+          <t>Which project it belongs to</t>
         </is>
       </c>
       <c r="G6" s="5" t="inlineStr">
@@ -1269,7 +1269,7 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Research Areas</t>
+          <t>Projects</t>
         </is>
       </c>
     </row>
@@ -1307,7 +1307,7 @@
     <row r="6" ht="58" customHeight="1">
       <c r="A6" s="5" t="inlineStr">
         <is>
-          <t>Name of the focus area</t>
+          <t>Name of the project</t>
         </is>
       </c>
       <c r="B6" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Replace Word member form with a Members tab in the workbook
- Delete Kuo-Lab-Member-Profile-Form.docx; everything is now one shareable
  Excel file
- Add a Members tab (Role, Name, Position, Project(s), About you, Email,
  Website, Scholar, CV) with a Role dropdown and a 3-4 sentence 'About you'
  field for personality
- Importer now reads Members into src/content/people/*.md: Role=PI writes
  kuo.md with role pi; email opt-out ('do not publish'/blank) omits the
  email; projects become interest tags; About you becomes the bio
- Update content-forms/README for the single-workbook workflow

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/content-forms/Kuo-Lab-Content-Workbook.xlsx
+++ b/content-forms/Kuo-Lab-Content-Workbook.xlsx
@@ -7,10 +7,11 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Publications" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Alumni" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="News" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Projects" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Members" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Publications" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Alumni" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="News" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Projects" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -491,6 +492,356 @@
   <dimension ref="A1:I22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="48" customWidth="1" min="5" max="5"/>
+    <col width="24" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="22" customWidth="1" min="8" max="8"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Members</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>The Kuo Lab — website content</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>One row per person — including the PI (set Role to 'PI'). Email your photo separately. The yellow row is an example — leave it or delete it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="22" customHeight="1">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Role</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="inlineStr">
+        <is>
+          <t>Name</t>
+        </is>
+      </c>
+      <c r="C5" s="4" t="inlineStr">
+        <is>
+          <t>Position</t>
+        </is>
+      </c>
+      <c r="D5" s="4" t="inlineStr">
+        <is>
+          <t>Project(s)</t>
+        </is>
+      </c>
+      <c r="E5" s="4" t="inlineStr">
+        <is>
+          <t>About you</t>
+        </is>
+      </c>
+      <c r="F5" s="4" t="inlineStr">
+        <is>
+          <t>Email</t>
+        </is>
+      </c>
+      <c r="G5" s="4" t="inlineStr">
+        <is>
+          <t>Website</t>
+        </is>
+      </c>
+      <c r="H5" s="4" t="inlineStr">
+        <is>
+          <t>Google Scholar</t>
+        </is>
+      </c>
+      <c r="I5" s="4" t="inlineStr">
+        <is>
+          <t>CV link</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="58" customHeight="1">
+      <c r="A6" s="5" t="inlineStr">
+        <is>
+          <t>Type 'Member' for everyone; 'PI' for the principal investigator</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="inlineStr">
+        <is>
+          <t>As you want it shown on the site</t>
+        </is>
+      </c>
+      <c r="C6" s="5" t="inlineStr">
+        <is>
+          <t>e.g. PhD Student, Postdoc, Lab Manager, Undergrad Researcher</t>
+        </is>
+      </c>
+      <c r="D6" s="5" t="inlineStr">
+        <is>
+          <t>Which project(s) you work on — list all that apply, separated by commas. Options: Gene Expression &amp; Regulation, Chromatin &amp; Epigenetics, Cell Growth &amp; Signaling</t>
+        </is>
+      </c>
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>3–4 sentences: your interests, what you're working on, and a bit of personality</t>
+        </is>
+      </c>
+      <c r="F6" s="5" t="inlineStr">
+        <is>
+          <t>Optional. Leave blank or write 'do not publish' to keep it off the site</t>
+        </is>
+      </c>
+      <c r="G6" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
+      <c r="I6" s="5" t="inlineStr">
+        <is>
+          <t>Optional (mainly for the PI) — link to a PDF</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="46" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>Member</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>Sam Park</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>PhD Student</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Chromatin &amp; Epigenetics</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>I study how cells package their DNA and what happens when that packaging goes wrong. Lately I've been using live-cell imaging to watch chromatin reorganize during division. Before grad school I worked in a plant genetics lab, and outside the lab I'm an avid rock climber.</t>
+        </is>
+      </c>
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>parksam@msu.edu</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr"/>
+      <c r="H7" s="6" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
+    </row>
+    <row r="8" ht="34" customHeight="1">
+      <c r="A8" s="7" t="inlineStr"/>
+      <c r="B8" s="7" t="inlineStr"/>
+      <c r="C8" s="7" t="inlineStr"/>
+      <c r="D8" s="7" t="inlineStr"/>
+      <c r="E8" s="7" t="inlineStr"/>
+      <c r="F8" s="7" t="inlineStr"/>
+      <c r="G8" s="7" t="inlineStr"/>
+      <c r="H8" s="7" t="inlineStr"/>
+      <c r="I8" s="7" t="inlineStr"/>
+    </row>
+    <row r="9" ht="34" customHeight="1">
+      <c r="A9" s="7" t="inlineStr"/>
+      <c r="B9" s="7" t="inlineStr"/>
+      <c r="C9" s="7" t="inlineStr"/>
+      <c r="D9" s="7" t="inlineStr"/>
+      <c r="E9" s="7" t="inlineStr"/>
+      <c r="F9" s="7" t="inlineStr"/>
+      <c r="G9" s="7" t="inlineStr"/>
+      <c r="H9" s="7" t="inlineStr"/>
+      <c r="I9" s="7" t="inlineStr"/>
+    </row>
+    <row r="10" ht="34" customHeight="1">
+      <c r="A10" s="7" t="inlineStr"/>
+      <c r="B10" s="7" t="inlineStr"/>
+      <c r="C10" s="7" t="inlineStr"/>
+      <c r="D10" s="7" t="inlineStr"/>
+      <c r="E10" s="7" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr"/>
+      <c r="G10" s="7" t="inlineStr"/>
+      <c r="H10" s="7" t="inlineStr"/>
+      <c r="I10" s="7" t="inlineStr"/>
+    </row>
+    <row r="11" ht="34" customHeight="1">
+      <c r="A11" s="7" t="inlineStr"/>
+      <c r="B11" s="7" t="inlineStr"/>
+      <c r="C11" s="7" t="inlineStr"/>
+      <c r="D11" s="7" t="inlineStr"/>
+      <c r="E11" s="7" t="inlineStr"/>
+      <c r="F11" s="7" t="inlineStr"/>
+      <c r="G11" s="7" t="inlineStr"/>
+      <c r="H11" s="7" t="inlineStr"/>
+      <c r="I11" s="7" t="inlineStr"/>
+    </row>
+    <row r="12" ht="34" customHeight="1">
+      <c r="A12" s="7" t="inlineStr"/>
+      <c r="B12" s="7" t="inlineStr"/>
+      <c r="C12" s="7" t="inlineStr"/>
+      <c r="D12" s="7" t="inlineStr"/>
+      <c r="E12" s="7" t="inlineStr"/>
+      <c r="F12" s="7" t="inlineStr"/>
+      <c r="G12" s="7" t="inlineStr"/>
+      <c r="H12" s="7" t="inlineStr"/>
+      <c r="I12" s="7" t="inlineStr"/>
+    </row>
+    <row r="13" ht="34" customHeight="1">
+      <c r="A13" s="7" t="inlineStr"/>
+      <c r="B13" s="7" t="inlineStr"/>
+      <c r="C13" s="7" t="inlineStr"/>
+      <c r="D13" s="7" t="inlineStr"/>
+      <c r="E13" s="7" t="inlineStr"/>
+      <c r="F13" s="7" t="inlineStr"/>
+      <c r="G13" s="7" t="inlineStr"/>
+      <c r="H13" s="7" t="inlineStr"/>
+      <c r="I13" s="7" t="inlineStr"/>
+    </row>
+    <row r="14" ht="34" customHeight="1">
+      <c r="A14" s="7" t="inlineStr"/>
+      <c r="B14" s="7" t="inlineStr"/>
+      <c r="C14" s="7" t="inlineStr"/>
+      <c r="D14" s="7" t="inlineStr"/>
+      <c r="E14" s="7" t="inlineStr"/>
+      <c r="F14" s="7" t="inlineStr"/>
+      <c r="G14" s="7" t="inlineStr"/>
+      <c r="H14" s="7" t="inlineStr"/>
+      <c r="I14" s="7" t="inlineStr"/>
+    </row>
+    <row r="15" ht="34" customHeight="1">
+      <c r="A15" s="7" t="inlineStr"/>
+      <c r="B15" s="7" t="inlineStr"/>
+      <c r="C15" s="7" t="inlineStr"/>
+      <c r="D15" s="7" t="inlineStr"/>
+      <c r="E15" s="7" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr"/>
+      <c r="G15" s="7" t="inlineStr"/>
+      <c r="H15" s="7" t="inlineStr"/>
+      <c r="I15" s="7" t="inlineStr"/>
+    </row>
+    <row r="16" ht="34" customHeight="1">
+      <c r="A16" s="7" t="inlineStr"/>
+      <c r="B16" s="7" t="inlineStr"/>
+      <c r="C16" s="7" t="inlineStr"/>
+      <c r="D16" s="7" t="inlineStr"/>
+      <c r="E16" s="7" t="inlineStr"/>
+      <c r="F16" s="7" t="inlineStr"/>
+      <c r="G16" s="7" t="inlineStr"/>
+      <c r="H16" s="7" t="inlineStr"/>
+      <c r="I16" s="7" t="inlineStr"/>
+    </row>
+    <row r="17" ht="34" customHeight="1">
+      <c r="A17" s="7" t="inlineStr"/>
+      <c r="B17" s="7" t="inlineStr"/>
+      <c r="C17" s="7" t="inlineStr"/>
+      <c r="D17" s="7" t="inlineStr"/>
+      <c r="E17" s="7" t="inlineStr"/>
+      <c r="F17" s="7" t="inlineStr"/>
+      <c r="G17" s="7" t="inlineStr"/>
+      <c r="H17" s="7" t="inlineStr"/>
+      <c r="I17" s="7" t="inlineStr"/>
+    </row>
+    <row r="18" ht="34" customHeight="1">
+      <c r="A18" s="7" t="inlineStr"/>
+      <c r="B18" s="7" t="inlineStr"/>
+      <c r="C18" s="7" t="inlineStr"/>
+      <c r="D18" s="7" t="inlineStr"/>
+      <c r="E18" s="7" t="inlineStr"/>
+      <c r="F18" s="7" t="inlineStr"/>
+      <c r="G18" s="7" t="inlineStr"/>
+      <c r="H18" s="7" t="inlineStr"/>
+      <c r="I18" s="7" t="inlineStr"/>
+    </row>
+    <row r="19" ht="34" customHeight="1">
+      <c r="A19" s="7" t="inlineStr"/>
+      <c r="B19" s="7" t="inlineStr"/>
+      <c r="C19" s="7" t="inlineStr"/>
+      <c r="D19" s="7" t="inlineStr"/>
+      <c r="E19" s="7" t="inlineStr"/>
+      <c r="F19" s="7" t="inlineStr"/>
+      <c r="G19" s="7" t="inlineStr"/>
+      <c r="H19" s="7" t="inlineStr"/>
+      <c r="I19" s="7" t="inlineStr"/>
+    </row>
+    <row r="20" ht="34" customHeight="1">
+      <c r="A20" s="7" t="inlineStr"/>
+      <c r="B20" s="7" t="inlineStr"/>
+      <c r="C20" s="7" t="inlineStr"/>
+      <c r="D20" s="7" t="inlineStr"/>
+      <c r="E20" s="7" t="inlineStr"/>
+      <c r="F20" s="7" t="inlineStr"/>
+      <c r="G20" s="7" t="inlineStr"/>
+      <c r="H20" s="7" t="inlineStr"/>
+      <c r="I20" s="7" t="inlineStr"/>
+    </row>
+    <row r="21" ht="34" customHeight="1">
+      <c r="A21" s="7" t="inlineStr"/>
+      <c r="B21" s="7" t="inlineStr"/>
+      <c r="C21" s="7" t="inlineStr"/>
+      <c r="D21" s="7" t="inlineStr"/>
+      <c r="E21" s="7" t="inlineStr"/>
+      <c r="F21" s="7" t="inlineStr"/>
+      <c r="G21" s="7" t="inlineStr"/>
+      <c r="H21" s="7" t="inlineStr"/>
+      <c r="I21" s="7" t="inlineStr"/>
+    </row>
+    <row r="22" ht="34" customHeight="1">
+      <c r="A22" s="7" t="inlineStr"/>
+      <c r="B22" s="7" t="inlineStr"/>
+      <c r="C22" s="7" t="inlineStr"/>
+      <c r="D22" s="7" t="inlineStr"/>
+      <c r="E22" s="7" t="inlineStr"/>
+      <c r="F22" s="7" t="inlineStr"/>
+      <c r="G22" s="7" t="inlineStr"/>
+      <c r="H22" s="7" t="inlineStr"/>
+      <c r="I22" s="7" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A3:I3"/>
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
+  <dataValidations count="1">
+    <dataValidation sqref="A8:A22" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Member,PI"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I22"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
     <col width="30" customWidth="1" min="2" max="2"/>
     <col width="26" customWidth="1" min="3" max="3"/>
@@ -848,7 +1199,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1050,7 +1401,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1252,7 +1603,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>